<commit_message>
feat: Add report for DeepWeeds classification and update results spreadsheet
</commit_message>
<xml_diff>
--- a/submissions/2A202602947_HoangTrungKhai/results.xlsx
+++ b/submissions/2A202602947_HoangTrungKhai/results.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -521,6 +521,236 @@
       <c r="M1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>a1_in1k</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>23.526473</v>
+      </c>
+      <c r="E2" t="n">
+        <v>4.087154688</v>
+      </c>
+      <c r="F2" t="n">
+        <v>224</v>
+      </c>
+      <c r="G2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.7742261482977252</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.834333047700657</v>
+      </c>
+      <c r="K2" t="n">
+        <v>57.20060948024994</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Single screening seed; latency not measured</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>resnext50_32x4d</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>a1h_in1k</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>22.998345</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4.228450304</v>
+      </c>
+      <c r="F3" t="n">
+        <v>224</v>
+      </c>
+      <c r="G3" t="n">
+        <v>7</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.6478821647382818</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.7529277349328763</v>
+      </c>
+      <c r="K3" t="n">
+        <v>54.15904277633346</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Single screening seed; latency not measured</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>in12k_ft_in1k</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4.454770176</v>
+      </c>
+      <c r="F4" t="n">
+        <v>224</v>
+      </c>
+      <c r="G4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.9694226904535661</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.9762924878606113</v>
+      </c>
+      <c r="K4" t="n">
+        <v>47.46537993883339</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Single screening seed; latency not measured</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>deit_small_patch16_224</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>fb_in1k</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>21.669129</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4.240838016</v>
+      </c>
+      <c r="F5" t="n">
+        <v>224</v>
+      </c>
+      <c r="G5" t="n">
+        <v>9</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.9511345493010324</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.9640102827763496</v>
+      </c>
+      <c r="K5" t="n">
+        <v>36.54267647916686</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Single screening seed; latency not measured</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>mobilenetv3_large_100</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ra_in1k</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.213561</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.21532128</v>
+      </c>
+      <c r="F6" t="n">
+        <v>224</v>
+      </c>
+      <c r="G6" t="n">
+        <v>12</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.6563820959585678</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.7589260211368181</v>
+      </c>
+      <c r="K6" t="n">
+        <v>31.71789946591646</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Single screening seed; latency not measured</t>
         </is>
       </c>
     </row>

</xml_diff>